<commit_message>
changed calculation of average pressure and burnrate, alongside other improvements
- Changed calculation of average pressure and burnrate: added another statistic that calculates average pressure and burnrate only for points where the pressure is higher than the average pressure calculated by the pressure integral over the whole fire. These new statistics are also saved in the output Excel spreadsheet and used for new calculation of a and n for the burn rate law.
- Added R^2 statistic for the power law fit for both characterization methods (old and new).
- Readability fixes and commenting.
- TODO: Clean up code and comments. Improve readability.
</commit_message>
<xml_diff>
--- a/characterization/out/out1/out1.xlsx
+++ b/characterization/out/out1/out1.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="0" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="2" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Characterization" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CharacterizationOld" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CharacterizationNew" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -727,7 +728,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Pressure Integral (MPa*s)</t>
+          <t>Full Pressure Integral (MPa*s)</t>
         </is>
       </c>
       <c r="T4" t="n">
@@ -855,7 +856,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Average Pressure (MPa)</t>
+          <t>Average Pressure (using full fire) (MPa)</t>
         </is>
       </c>
       <c r="T6" t="n">
@@ -919,11 +920,11 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Average Burnrate (mm/s)</t>
+          <t>Average Burnrate (using full fire) (mm/s)</t>
         </is>
       </c>
       <c r="T7" t="n">
-        <v>4.05402973936427</v>
+        <v>4.041832530086078</v>
       </c>
     </row>
     <row r="8">
@@ -983,11 +984,11 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Impulse (lbf*s)</t>
+          <t>Average Pressure (using points above average) (MPa)</t>
         </is>
       </c>
       <c r="T8" t="n">
-        <v>287.1698168739581</v>
+        <v>2.763920541652142</v>
       </c>
     </row>
     <row r="9">
@@ -1047,11 +1048,11 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Pressure Integral (psig*s)</t>
+          <t>Average Burnrate (using points above average) (mm/s)</t>
         </is>
       </c>
       <c r="T9" t="n">
-        <v>993.3487485792778</v>
+        <v>5.111268030844618</v>
       </c>
     </row>
     <row r="10">
@@ -1111,11 +1112,11 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>C* (ft/s)</t>
+          <t>Impulse (lbf*s)</t>
         </is>
       </c>
       <c r="T10" t="n">
-        <v>4906.967022018958</v>
+        <v>287.1698168739581</v>
       </c>
     </row>
     <row r="11">
@@ -1175,11 +1176,11 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Average Pressure (psig)</t>
+          <t>Full Pressure Integral (psig*s)</t>
         </is>
       </c>
       <c r="T11" t="n">
-        <v>314.3508698035691</v>
+        <v>993.3487485792778</v>
       </c>
     </row>
     <row r="12">
@@ -1239,11 +1240,11 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Average Burnrate (in/s)</t>
+          <t>C* (ft/s)</t>
         </is>
       </c>
       <c r="T12" t="n">
-        <v>0.1596075562417453</v>
+        <v>4906.967022018958</v>
       </c>
     </row>
     <row r="13">
@@ -1303,11 +1304,11 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>ISP (sec)</t>
+          <t>Average Pressure (using full fire) (psig)</t>
         </is>
       </c>
       <c r="T13" t="n">
-        <v>188.2438775450109</v>
+        <v>314.3508698035691</v>
       </c>
     </row>
     <row r="14">
@@ -1365,8 +1366,14 @@
       <c r="R14" t="n">
         <v>0.1831493679691062</v>
       </c>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr"/>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Average Burnrate (in/s) (using full fire)</t>
+        </is>
+      </c>
+      <c r="T14" t="n">
+        <v>0.1591273508927419</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -1423,8 +1430,14 @@
       <c r="R15" t="n">
         <v>0.1861325971301015</v>
       </c>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Average Pressure (using points above average) (psig)</t>
+        </is>
+      </c>
+      <c r="T15" t="n">
+        <v>400.8727826267029</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -1481,8 +1494,14 @@
       <c r="R16" t="n">
         <v>0.186503166492563</v>
       </c>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Average Burnrate (using points above average) (in/s)</t>
+        </is>
+      </c>
+      <c r="T16" t="n">
+        <v>0.2012311335011557</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -1539,8 +1558,14 @@
       <c r="R17" t="n">
         <v>0.1882038398130086</v>
       </c>
-      <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>ISP (sec)</t>
+        </is>
+      </c>
+      <c r="T17" t="n">
+        <v>188.2438775450109</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -5260,7 +5285,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Pressure Integral (MPa*s)</t>
+          <t>Full Pressure Integral (MPa*s)</t>
         </is>
       </c>
       <c r="T4" t="n">
@@ -5388,7 +5413,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Average Pressure (MPa)</t>
+          <t>Average Pressure (using full fire) (MPa)</t>
         </is>
       </c>
       <c r="T6" t="n">
@@ -5452,11 +5477,11 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Average Burnrate (mm/s)</t>
+          <t>Average Burnrate (using full fire) (mm/s)</t>
         </is>
       </c>
       <c r="T7" t="n">
-        <v>4.18334586539266</v>
+        <v>4.254978472732983</v>
       </c>
     </row>
     <row r="8">
@@ -5516,11 +5541,11 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Impulse (lbf*s)</t>
+          <t>Average Pressure (using points above average) (MPa)</t>
         </is>
       </c>
       <c r="T8" t="n">
-        <v>280.2944475423513</v>
+        <v>3.248606501539229</v>
       </c>
     </row>
     <row r="9">
@@ -5580,11 +5605,11 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Pressure Integral (psig*s)</t>
+          <t>Average Burnrate (using points above average) (mm/s)</t>
         </is>
       </c>
       <c r="T9" t="n">
-        <v>1092.014030435683</v>
+        <v>5.408119403133058</v>
       </c>
     </row>
     <row r="10">
@@ -5644,11 +5669,11 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>C* (ft/s)</t>
+          <t>Impulse (lbf*s)</t>
         </is>
       </c>
       <c r="T10" t="n">
-        <v>5102.034198575786</v>
+        <v>280.2944475423513</v>
       </c>
     </row>
     <row r="11">
@@ -5708,11 +5733,11 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Average Pressure (psig)</t>
+          <t>Full Pressure Integral (psig*s)</t>
         </is>
       </c>
       <c r="T11" t="n">
-        <v>363.7621686994284</v>
+        <v>1092.014030435683</v>
       </c>
     </row>
     <row r="12">
@@ -5772,11 +5797,11 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Average Burnrate (in/s)</t>
+          <t>C* (ft/s)</t>
         </is>
       </c>
       <c r="T12" t="n">
-        <v>0.1646987450550956</v>
+        <v>5102.034198575786</v>
       </c>
     </row>
     <row r="13">
@@ -5836,11 +5861,11 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>ISP (sec)</t>
+          <t>Average Pressure (using full fire) (psig)</t>
         </is>
       </c>
       <c r="T13" t="n">
-        <v>183.7369756824667</v>
+        <v>363.7621686994284</v>
       </c>
     </row>
     <row r="14">
@@ -5898,8 +5923,14 @@
       <c r="R14" t="n">
         <v>0.1691730481724457</v>
       </c>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr"/>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Average Burnrate (in/s) (using full fire)</t>
+        </is>
+      </c>
+      <c r="T14" t="n">
+        <v>0.1675189279693448</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -5956,8 +5987,14 @@
       <c r="R15" t="n">
         <v>0.1729375470320409</v>
       </c>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Average Pressure (using points above average) (psig)</t>
+        </is>
+      </c>
+      <c r="T15" t="n">
+        <v>471.1705377582196</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -6014,8 +6051,14 @@
       <c r="R16" t="n">
         <v>0.1753736013128037</v>
       </c>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Average Burnrate (using points above average) (in/s)</t>
+        </is>
+      </c>
+      <c r="T16" t="n">
+        <v>0.2129182017132888</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -6072,8 +6115,14 @@
       <c r="R17" t="n">
         <v>0.1785005451706855</v>
       </c>
-      <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>ISP (sec)</t>
+        </is>
+      </c>
+      <c r="T17" t="n">
+        <v>183.7369756824667</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -9561,7 +9610,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>Pressure Integral (MPa*s)</t>
+          <t>Full Pressure Integral (MPa*s)</t>
         </is>
       </c>
       <c r="T4" t="n">
@@ -9689,7 +9738,7 @@
       </c>
       <c r="S6" t="inlineStr">
         <is>
-          <t>Average Pressure (MPa)</t>
+          <t>Average Pressure (using full fire) (MPa)</t>
         </is>
       </c>
       <c r="T6" t="n">
@@ -9753,11 +9802,11 @@
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Average Burnrate (mm/s)</t>
+          <t>Average Burnrate (using full fire) (mm/s)</t>
         </is>
       </c>
       <c r="T7" t="n">
-        <v>4.30999455351504</v>
+        <v>4.302532935072866</v>
       </c>
     </row>
     <row r="8">
@@ -9817,11 +9866,11 @@
       </c>
       <c r="S8" t="inlineStr">
         <is>
-          <t>Impulse (lbf*s)</t>
+          <t>Average Pressure (using points above average) (MPa)</t>
         </is>
       </c>
       <c r="T8" t="n">
-        <v>289.3762587523703</v>
+        <v>3.546304583953522</v>
       </c>
     </row>
     <row r="9">
@@ -9881,11 +9930,11 @@
       </c>
       <c r="S9" t="inlineStr">
         <is>
-          <t>Pressure Integral (psig*s)</t>
+          <t>Average Burnrate (using points above average) (mm/s)</t>
         </is>
       </c>
       <c r="T9" t="n">
-        <v>1155.231503595463</v>
+        <v>5.581836910624572</v>
       </c>
     </row>
     <row r="10">
@@ -9945,11 +9994,11 @@
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>C* (ft/s)</t>
+          <t>Impulse (lbf*s)</t>
         </is>
       </c>
       <c r="T10" t="n">
-        <v>5077.028328865798</v>
+        <v>289.3762587523703</v>
       </c>
     </row>
     <row r="11">
@@ -10009,11 +10058,11 @@
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Average Pressure (psig)</t>
+          <t>Full Pressure Integral (psig*s)</t>
         </is>
       </c>
       <c r="T11" t="n">
-        <v>389.0978456030527</v>
+        <v>1155.231503595463</v>
       </c>
     </row>
     <row r="12">
@@ -10073,11 +10122,11 @@
       </c>
       <c r="S12" t="inlineStr">
         <is>
-          <t>Average Burnrate (in/s)</t>
+          <t>C* (ft/s)</t>
         </is>
       </c>
       <c r="T12" t="n">
-        <v>0.1696849165713425</v>
+        <v>5077.028328865798</v>
       </c>
     </row>
     <row r="13">
@@ -10137,11 +10186,11 @@
       </c>
       <c r="S13" t="inlineStr">
         <is>
-          <t>ISP (sec)</t>
+          <t>Average Pressure (using full fire) (psig)</t>
         </is>
       </c>
       <c r="T13" t="n">
-        <v>189.6902314107875</v>
+        <v>389.0978456030527</v>
       </c>
     </row>
     <row r="14">
@@ -10199,8 +10248,14 @@
       <c r="R14" t="n">
         <v>0.1574542322366897</v>
       </c>
-      <c r="S14" t="inlineStr"/>
-      <c r="T14" t="inlineStr"/>
+      <c r="S14" t="inlineStr">
+        <is>
+          <t>Average Burnrate (in/s) (using full fire)</t>
+        </is>
+      </c>
+      <c r="T14" t="n">
+        <v>0.1693911519071123</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -10257,8 +10312,14 @@
       <c r="R15" t="n">
         <v>0.1612236363779067</v>
       </c>
-      <c r="S15" t="inlineStr"/>
-      <c r="T15" t="inlineStr"/>
+      <c r="S15" t="inlineStr">
+        <is>
+          <t>Average Pressure (using points above average) (psig)</t>
+        </is>
+      </c>
+      <c r="T15" t="n">
+        <v>514.3479941581477</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -10315,8 +10376,14 @@
       <c r="R16" t="n">
         <v>0.1642047448147796</v>
       </c>
-      <c r="S16" t="inlineStr"/>
-      <c r="T16" t="inlineStr"/>
+      <c r="S16" t="inlineStr">
+        <is>
+          <t>Average Burnrate (using points above average) (in/s)</t>
+        </is>
+      </c>
+      <c r="T16" t="n">
+        <v>0.2197574773549804</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -10373,8 +10440,14 @@
       <c r="R17" t="n">
         <v>0.1679482796174904</v>
       </c>
-      <c r="S17" t="inlineStr"/>
-      <c r="T17" t="inlineStr"/>
+      <c r="S17" t="inlineStr">
+        <is>
+          <t>ISP (sec)</t>
+        </is>
+      </c>
+      <c r="T17" t="n">
+        <v>189.6902314107875</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -13519,7 +13592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -13555,7 +13628,7 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>3.264517615750071</v>
+        <v>3.208067467435161</v>
       </c>
     </row>
     <row r="4">
@@ -13568,7 +13641,7 @@
         </is>
       </c>
       <c r="C4" t="n">
-        <v>0.2770474995445706</v>
+        <v>0.3011424723224058</v>
       </c>
     </row>
     <row r="5">
@@ -13592,7 +13665,7 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>0.03237073898836026</v>
+        <v>0.0282160557422733</v>
       </c>
     </row>
     <row r="7">
@@ -13605,7 +13678,155 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>0.2770475031812422</v>
+        <v>0.3011424601959523</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>R^2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.9778325083573611</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>str</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>dat</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Metric (MPa and mm):</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>3.569521401001583</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>0.3529753624705195</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Imperial (psig and in):</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>a</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>0.02425643444460022</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>0.3529753624981126</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t xml:space="preserve"> </t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>R^2</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>0.999931783880587</v>
       </c>
     </row>
   </sheetData>

</xml_diff>